<commit_message>
Add SOH report for 2026-10-10
</commit_message>
<xml_diff>
--- a/reports/SOH_09_10_2026.xlsx
+++ b/reports/SOH_09_10_2026.xlsx
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>21000</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1</v>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>-32</v>
+        <v>-33</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>8000</v>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>528</v>
+        <v>524</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>25000</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1144</v>
+        <v>1139</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>40000</v>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>10500</v>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>48000</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>367</v>
+        <v>354</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>10500</v>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="E40" s="3" t="n">
         <v>21000</v>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>622</v>
+        <v>612</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>4500</v>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1066</v>
+        <v>1063</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>12500</v>
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E49" s="3" t="n">
         <v>81000</v>
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>459</v>
+        <v>452</v>
       </c>
       <c r="E53" s="3" t="n">
         <v>81000</v>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1312</v>
+        <v>1308</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>51000</v>
@@ -2417,11 +2417,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>AIWIBI Baby Short Sleevet-Shirt (12-24M)</t>
+          <t>AIWIBI Baby Short Sleevet-Shirt (12-18M)</t>
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E71" s="3" t="n">
         <v>1</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E72" s="3" t="n">
         <v>1</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>4000</v>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E102" s="3" t="n">
         <v>4708</v>
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E108" s="3" t="n">
         <v>1</v>
@@ -3485,7 +3485,7 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>2891</v>
+        <v>2890</v>
       </c>
       <c r="E109" s="3" t="n">
         <v>3876</v>
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>4807</v>
+        <v>4803</v>
       </c>
       <c r="E126" s="3" t="n">
         <v>2500</v>
@@ -4685,7 +4685,7 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E152" s="3" t="n">
         <v>1</v>
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E155" s="3" t="n">
         <v>1</v>
@@ -4797,7 +4797,7 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="E156" s="3" t="n">
         <v>26000</v>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>478</v>
+        <v>456</v>
       </c>
       <c r="E157" s="3" t="n">
         <v>1</v>
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="E159" s="3" t="n">
         <v>1</v>
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E168" s="3" t="n">
         <v>1</v>
@@ -5493,7 +5493,7 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E182" s="3" t="n">
         <v>1</v>
@@ -6177,7 +6177,7 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E207" s="3" t="n">
         <v>1</v>
@@ -6511,52 +6511,48 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>8017123451008</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>ASBH</t>
+          <t>API040</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>AWB Sweet Beginnings Hamper</t>
+          <t>AWB SUNSHADE UMBRELLA-OUTDOOR</t>
         </is>
       </c>
       <c r="D220" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E220" s="3" t="n">
-        <v>38880</v>
-      </c>
-      <c r="F220" t="inlineStr">
-        <is>
-          <t>AIWIBI</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>8017123451046</t>
+          <t>8017123451008</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>AUWH</t>
+          <t>ASBH</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>AWB Ultimate Welcome Hamper</t>
+          <t>AWB Sweet Beginnings Hamper</t>
         </is>
       </c>
       <c r="D221" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E221" s="3" t="n">
-        <v>253035</v>
+        <v>38880</v>
       </c>
       <c r="F221" t="inlineStr">
         <is>
@@ -6591,24 +6587,24 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8017123451046</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>API065</t>
+          <t>AUWH</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>AWB UMBRELLA</t>
+          <t>AWB Ultimate Welcome Hamper</t>
         </is>
       </c>
       <c r="D223" s="2" t="n">
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="E223" s="3" t="n">
-        <v>1</v>
+        <v>253035</v>
       </c>
       <c r="F223" t="inlineStr">
         <is>
@@ -6624,21 +6620,25 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>API040</t>
+          <t>API065</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>AWB SUNSHADE UMBRELLA-OUTDOOR</t>
+          <t>AWB UMBRELLA</t>
         </is>
       </c>
       <c r="D224" s="2" t="n">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="E224" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F224" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>AIWIBI</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -6685,7 +6685,7 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="E226" s="3" t="n">
         <v>1</v>
@@ -9177,7 +9177,7 @@
         </is>
       </c>
       <c r="D316" s="2" t="n">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="E316" s="3" t="n">
         <v>39894</v>
@@ -9289,7 +9289,7 @@
         </is>
       </c>
       <c r="D320" s="2" t="n">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E320" s="3" t="n">
         <v>16171</v>
@@ -10074,7 +10074,7 @@
         </is>
       </c>
       <c r="D348" s="2" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E348" s="3" t="n">
         <v>50976</v>
@@ -10186,7 +10186,7 @@
         </is>
       </c>
       <c r="D352" s="2" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E352" s="3" t="n">
         <v>31328</v>
@@ -12664,24 +12664,24 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>5060677904907</t>
+          <t>5060677903528</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>90490</t>
+          <t>90352</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>CHUPA CHUPS 18OZ JAR CANDLE MA</t>
+          <t>CHUPA CHUPS 18OZ JAR CANDLE CH</t>
         </is>
       </c>
       <c r="D441" s="2" t="n">
-        <v>366</v>
+        <v>319</v>
       </c>
       <c r="E441" s="3" t="n">
-        <v>37709</v>
+        <v>37711</v>
       </c>
       <c r="F441" t="inlineStr">
         <is>
@@ -12720,24 +12720,24 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>5060677903535</t>
+          <t>5060677904907</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>90353</t>
+          <t>90490</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>CHUPA CHUPS 18OZ JAR CANDLE ST</t>
+          <t>CHUPA CHUPS 18OZ JAR CANDLE MA</t>
         </is>
       </c>
       <c r="D443" s="2" t="n">
-        <v>312</v>
+        <v>366</v>
       </c>
       <c r="E443" s="3" t="n">
-        <v>37711</v>
+        <v>37709</v>
       </c>
       <c r="F443" t="inlineStr">
         <is>
@@ -12748,24 +12748,24 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>5060677909148</t>
+          <t>5060677903535</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>90910</t>
+          <t>90353</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>CHUPA CHUPS AIR FRESHENER SCEN</t>
+          <t>CHUPA CHUPS 18OZ JAR CANDLE ST</t>
         </is>
       </c>
       <c r="D444" s="2" t="n">
-        <v>71</v>
+        <v>312</v>
       </c>
       <c r="E444" s="3" t="n">
-        <v>8734</v>
+        <v>37711</v>
       </c>
       <c r="F444" t="inlineStr">
         <is>
@@ -12776,24 +12776,24 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>5060677903528</t>
+          <t>5060677909148</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>90352</t>
+          <t>90910</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>CHUPA CHUPS 18OZ JAR CANDLE CH</t>
+          <t>CHUPA CHUPS AIR FRESHENER SCEN</t>
         </is>
       </c>
       <c r="D445" s="2" t="n">
-        <v>319</v>
+        <v>71</v>
       </c>
       <c r="E445" s="3" t="n">
-        <v>37711</v>
+        <v>8734</v>
       </c>
       <c r="F445" t="inlineStr">
         <is>
@@ -12874,7 +12874,7 @@
         </is>
       </c>
       <c r="D448" s="2" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E448" s="3" t="n">
         <v>8856</v>
@@ -16976,24 +16976,24 @@
     <row r="595">
       <c r="A595" t="inlineStr">
         <is>
-          <t>9333527598813</t>
+          <t>9333527144508</t>
         </is>
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>BC0603</t>
+          <t>BB0030</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
         <is>
-          <t>ECO FRIENDLY CLEANING CLOTH 2P</t>
+          <t>DUSTPAN N BRUSH SILVER/BLACK</t>
         </is>
       </c>
       <c r="D595" s="2" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="E595" s="3" t="n">
-        <v>13122</v>
+        <v>13111</v>
       </c>
       <c r="F595" t="inlineStr">
         <is>
@@ -17004,24 +17004,24 @@
     <row r="596">
       <c r="A596" t="inlineStr">
         <is>
-          <t>9333527598820</t>
+          <t>9333527006356</t>
         </is>
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>BC0604</t>
+          <t>ER0005</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
         <is>
-          <t>ECO FRIENDLY CLEANING SPONGE 2</t>
+          <t>DVD CASE SLIMLINE 7PK</t>
         </is>
       </c>
       <c r="D596" s="2" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="E596" s="3" t="n">
-        <v>14261</v>
+        <v>9901</v>
       </c>
       <c r="F596" t="inlineStr">
         <is>
@@ -17032,24 +17032,24 @@
     <row r="597">
       <c r="A597" t="inlineStr">
         <is>
-          <t>9333527662286</t>
+          <t>9333527598813</t>
         </is>
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>AG4607</t>
+          <t>BC0603</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>ECO RAZOR W/3 BLADES 4 PACK</t>
+          <t>ECO FRIENDLY CLEANING CLOTH 2P</t>
         </is>
       </c>
       <c r="D597" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E597" s="3" t="n">
-        <v>13646</v>
+        <v>13122</v>
       </c>
       <c r="F597" t="inlineStr">
         <is>
@@ -17060,24 +17060,24 @@
     <row r="598">
       <c r="A598" t="inlineStr">
         <is>
-          <t>9333527006356</t>
+          <t>9333527598820</t>
         </is>
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>ER0005</t>
+          <t>BC0604</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
         <is>
-          <t>DVD CASE SLIMLINE 7PK</t>
+          <t>ECO FRIENDLY CLEANING SPONGE 2</t>
         </is>
       </c>
       <c r="D598" s="2" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="E598" s="3" t="n">
-        <v>9901</v>
+        <v>14261</v>
       </c>
       <c r="F598" t="inlineStr">
         <is>
@@ -17088,24 +17088,24 @@
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>9333527144508</t>
+          <t>9333527662286</t>
         </is>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>BB0030</t>
+          <t>AG4607</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>DUSTPAN N BRUSH SILVER/BLACK</t>
+          <t>ECO RAZOR W/3 BLADES 4 PACK</t>
         </is>
       </c>
       <c r="D599" s="2" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="E599" s="3" t="n">
-        <v>13111</v>
+        <v>13646</v>
       </c>
       <c r="F599" t="inlineStr">
         <is>
@@ -18111,7 +18111,7 @@
         </is>
       </c>
       <c r="D635" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E635" s="3" t="n">
         <v>42078</v>
@@ -18895,7 +18895,7 @@
         </is>
       </c>
       <c r="D663" s="2" t="n">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E663" s="3" t="n">
         <v>3987</v>
@@ -21009,24 +21009,24 @@
     <row r="739">
       <c r="A739" t="inlineStr">
         <is>
-          <t>9333527522214</t>
+          <t>9333527730121</t>
         </is>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>AH3664</t>
+          <t>AH5286</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>HAIR BRUSH PADDLE ROSE GOLD</t>
+          <t>HAIR BRUSH PADDLE BLACK</t>
         </is>
       </c>
       <c r="D739" s="2" t="n">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="E739" s="3" t="n">
-        <v>0</v>
+        <v>16972</v>
       </c>
       <c r="F739" t="inlineStr">
         <is>
@@ -21037,24 +21037,24 @@
     <row r="740">
       <c r="A740" t="inlineStr">
         <is>
-          <t>9333527803931</t>
+          <t>9333527522214</t>
         </is>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>AH0000074</t>
+          <t>AH3664</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>HAIR CLAW CLIP LARGE 1 PIECE 3 ASSORTED</t>
+          <t>HAIR BRUSH PADDLE ROSE GOLD</t>
         </is>
       </c>
       <c r="D740" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E740" s="3" t="n">
-        <v>17779</v>
+        <v>0</v>
       </c>
       <c r="F740" t="inlineStr">
         <is>
@@ -21093,24 +21093,24 @@
     <row r="742">
       <c r="A742" t="inlineStr">
         <is>
-          <t>9333527811127</t>
+          <t>9333527803931</t>
         </is>
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>AH0000128</t>
+          <t>AH0000074</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>HAIR CLAW CLIP PEARL LOOK 2 ASSORTED</t>
+          <t>HAIR CLAW CLIP LARGE 1 PIECE 3 ASSORTED</t>
         </is>
       </c>
       <c r="D742" s="2" t="n">
-        <v>87</v>
+        <v>20</v>
       </c>
       <c r="E742" s="3" t="n">
-        <v>7285</v>
+        <v>17779</v>
       </c>
       <c r="F742" t="inlineStr">
         <is>
@@ -21121,24 +21121,24 @@
     <row r="743">
       <c r="A743" t="inlineStr">
         <is>
-          <t>9333527730121</t>
+          <t>9333527811127</t>
         </is>
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>AH5286</t>
+          <t>AH0000128</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>HAIR BRUSH PADDLE BLACK</t>
+          <t>HAIR CLAW CLIP PEARL LOOK 2 ASSORTED</t>
         </is>
       </c>
       <c r="D743" s="2" t="n">
-        <v>192</v>
+        <v>87</v>
       </c>
       <c r="E743" s="3" t="n">
-        <v>16972</v>
+        <v>7285</v>
       </c>
       <c r="F743" t="inlineStr">
         <is>
@@ -23712,7 +23712,7 @@
         </is>
       </c>
       <c r="D835" s="2" t="n">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E835" s="3" t="n">
         <v>17750</v>
@@ -28588,7 +28588,7 @@
         </is>
       </c>
       <c r="D1009" s="2" t="n">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="E1009" s="3" t="n">
         <v>5243</v>
@@ -39705,7 +39705,7 @@
         </is>
       </c>
       <c r="D1406" s="2" t="n">
-        <v>1858</v>
+        <v>1857</v>
       </c>
       <c r="E1406" s="3" t="n">
         <v>11094</v>
@@ -40503,24 +40503,24 @@
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
-          <t>9333527779113</t>
+          <t>9333527779137</t>
         </is>
       </c>
       <c r="B1435" t="inlineStr">
         <is>
-          <t>KS0000139</t>
+          <t>KS0000140</t>
         </is>
       </c>
       <c r="C1435" t="inlineStr">
         <is>
-          <t>STORAGE JAR RIBBED WITH LID 1500ML</t>
+          <t>STORAGE JAR RIBBED WITH LID 1200ML</t>
         </is>
       </c>
       <c r="D1435" s="2" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="E1435" s="3" t="n">
-        <v>32556</v>
+        <v>28273</v>
       </c>
       <c r="F1435" t="inlineStr">
         <is>
@@ -40531,24 +40531,24 @@
     <row r="1436">
       <c r="A1436" t="inlineStr">
         <is>
-          <t>9333527779151</t>
+          <t>9333527779113</t>
         </is>
       </c>
       <c r="B1436" t="inlineStr">
         <is>
-          <t>KS0000141</t>
+          <t>KS0000139</t>
         </is>
       </c>
       <c r="C1436" t="inlineStr">
         <is>
-          <t>STORAGE JAR RIBBED WITH LID 800ML</t>
+          <t>STORAGE JAR RIBBED WITH LID 1500ML</t>
         </is>
       </c>
       <c r="D1436" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E1436" s="3" t="n">
-        <v>24631</v>
+        <v>32556</v>
       </c>
       <c r="F1436" t="inlineStr">
         <is>
@@ -40559,24 +40559,24 @@
     <row r="1437">
       <c r="A1437" t="inlineStr">
         <is>
-          <t>9333527779137</t>
+          <t>9333527779151</t>
         </is>
       </c>
       <c r="B1437" t="inlineStr">
         <is>
-          <t>KS0000140</t>
+          <t>KS0000141</t>
         </is>
       </c>
       <c r="C1437" t="inlineStr">
         <is>
-          <t>STORAGE JAR RIBBED WITH LID 1200ML</t>
+          <t>STORAGE JAR RIBBED WITH LID 800ML</t>
         </is>
       </c>
       <c r="D1437" s="2" t="n">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="E1437" s="3" t="n">
-        <v>28273</v>
+        <v>24631</v>
       </c>
       <c r="F1437" t="inlineStr">
         <is>
@@ -41189,7 +41189,7 @@
         </is>
       </c>
       <c r="D1459" s="2" t="n">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E1459" s="3" t="n">
         <v>15250</v>
@@ -41245,7 +41245,7 @@
         </is>
       </c>
       <c r="D1461" s="2" t="n">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E1461" s="3" t="n">
         <v>11283</v>
@@ -41749,7 +41749,7 @@
         </is>
       </c>
       <c r="D1479" s="2" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E1479" s="3" t="n">
         <v>7390</v>

</xml_diff>